<commit_message>
avance en la automatizaicón de graficos
</commit_message>
<xml_diff>
--- a/Backend/Input/ADP/Monitoreo ADP - Nivel I.xlsx
+++ b/Backend/Input/ADP/Monitoreo ADP - Nivel I.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mineduca.sharepoint.com/sites/PCG/Documentos compartidos/Reporte mensual -ATMM/ADP/Nivel I/2025/Abril/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mineduca.sharepoint.com/sites/PCG/Documentos compartidos/Reporte mensual -ATMM/ADP/Nivel I/2025/Mayo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="144" documentId="8_{50EE1512-5B22-4D40-BDDF-5CEBD82B5728}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3C1F4DD6-C869-4BB9-821E-7D45BDCF8A23}"/>
+  <xr:revisionPtr revIDLastSave="198" documentId="8_{50EE1512-5B22-4D40-BDDF-5CEBD82B5728}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{058233BB-EDA1-4860-BF84-2C76331E3007}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-4830" windowWidth="29040" windowHeight="15840" xr2:uid="{4A0AD951-A275-4FB5-B4BD-A57A3ECB8FBA}"/>
+    <workbookView xWindow="20370" yWindow="-3945" windowWidth="29040" windowHeight="15840" xr2:uid="{4A0AD951-A275-4FB5-B4BD-A57A3ECB8FBA}"/>
   </bookViews>
   <sheets>
     <sheet name="Fechas y comentarios" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="26">
   <si>
     <t>Servicio</t>
   </si>
@@ -83,9 +83,6 @@
     <t>Superintendencia de Educación Superior</t>
   </si>
   <si>
-    <t>ABRIL</t>
-  </si>
-  <si>
     <t>Comentarios</t>
   </si>
   <si>
@@ -98,16 +95,26 @@
     <t>En marzo 2025 se envió mediante mail del Jefe del Gabinete del Ministro, el resultado del monitoreo del tercer año de gestión.</t>
   </si>
   <si>
-    <t>En enero 2025 se tramitó totalmente el acto administrativo que aprueba el grado de cumplimiento global de las metas del convenio del segundo año de gestión.</t>
-  </si>
-  <si>
-    <t>En abril 2025 se envió mediante mail del Jefe del Gabinete del Ministro, el resultado del monitoreo del primer año de gestión.</t>
-  </si>
-  <si>
     <t>En febrero 2025 se tramitó totalmente el acto administrativo que aprueba el grado de cumplimiento global de las metas del convenio del segundo año de gestión.</t>
   </si>
   <si>
     <t>En abril 2025 se tramitó totalmente el acto administrativo que aprueba el grado de cumplimiento global de las metas del convenio del segundo año de gestión.</t>
+  </si>
+  <si>
+    <t>MAYO</t>
+  </si>
+  <si>
+    <t>Actualizado al 03.06.25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En mayo 2025 se inició el monitoreo del tercer año de gestión
+</t>
+  </si>
+  <si>
+    <t>En mayo 2025 se inició el proceso de evaluación del primer año de gestión.</t>
+  </si>
+  <si>
+    <t>En mayo 2025 se envió a tramitación el acto administrativo que aprueba el grado de cumplimiento global de las metas del convenio del segundo año de gestión.</t>
   </si>
 </sst>
 </file>
@@ -168,7 +175,6 @@
     </font>
     <font>
       <sz val="12"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -413,7 +419,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -753,7 +759,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="52" customWidth="1"/>
-    <col min="3" max="3" width="36.7109375" customWidth="1"/>
+    <col min="3" max="3" width="43.140625" customWidth="1"/>
     <col min="4" max="4" width="25.42578125" customWidth="1"/>
     <col min="5" max="5" width="25.85546875" customWidth="1"/>
     <col min="6" max="6" width="24.140625" customWidth="1"/>
@@ -860,7 +866,7 @@
       <c r="G7" s="7">
         <v>45599</v>
       </c>
-      <c r="H7" s="6">
+      <c r="H7" s="7">
         <v>45780</v>
       </c>
       <c r="I7" s="11">
@@ -877,7 +883,7 @@
       <c r="D8" s="5">
         <v>45623</v>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="5">
         <v>45804</v>
       </c>
       <c r="F8" s="6">
@@ -898,25 +904,25 @@
         <v>12</v>
       </c>
       <c r="C9" s="5">
-        <v>44900</v>
+        <v>45017</v>
       </c>
       <c r="D9" s="5">
-        <v>45082</v>
+        <v>45200</v>
       </c>
       <c r="E9" s="5">
-        <v>45265</v>
+        <v>45383</v>
       </c>
       <c r="F9" s="5">
-        <v>45448</v>
+        <v>45566</v>
       </c>
       <c r="G9" s="5">
-        <v>45631</v>
+        <v>45748</v>
       </c>
       <c r="H9" s="6">
-        <v>45813</v>
+        <v>45931</v>
       </c>
       <c r="I9" s="11">
-        <v>45813</v>
+        <v>46113</v>
       </c>
     </row>
     <row r="10" spans="2:9" ht="21" x14ac:dyDescent="0.25">
@@ -973,7 +979,7 @@
     </row>
     <row r="13" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C13" s="16" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14" spans="2:9" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -981,7 +987,7 @@
         <v>0</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" spans="2:9" ht="110.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -989,11 +995,11 @@
         <v>8</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D15" s="15"/>
       <c r="E15" s="18" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F15" s="4"/>
     </row>
@@ -1002,71 +1008,71 @@
         <v>9</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D16" s="15"/>
       <c r="E16" s="18" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="17" spans="2:5" ht="125.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" ht="56.25" x14ac:dyDescent="0.25">
       <c r="B17" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D17" s="15"/>
       <c r="E17" s="18" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="18" spans="2:5" ht="93.75" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" ht="37.5" x14ac:dyDescent="0.25">
       <c r="B18" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D18" s="15"/>
       <c r="E18" s="18" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="19" spans="2:5" ht="112.5" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" ht="93.75" x14ac:dyDescent="0.25">
       <c r="B19" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D19" s="15"/>
       <c r="E19" s="18" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="20" spans="2:5" ht="112.5" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" ht="93.75" x14ac:dyDescent="0.25">
       <c r="B20" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C20" s="17" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D20" s="15"/>
       <c r="E20" s="18" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="21" spans="2:5" ht="112.5" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" ht="93.75" x14ac:dyDescent="0.25">
       <c r="B21" s="12" t="s">
         <v>14</v>
       </c>
       <c r="C21" s="17" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D21" s="15"/>
       <c r="E21" s="18" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>